<commit_message>
Fix dashboard chart label
</commit_message>
<xml_diff>
--- a/Call_Center_Performance_Dashboard.xlsx
+++ b/Call_Center_Performance_Dashboard.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f82d214c28a4fdb9/Desktop/EXCEL Portfolio Projects/01-Excel-Call-Center-Dashboard/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/F82D214C28A4FDB9/Desktop/EXCEL Portfolio Projects/01-Excel-Call-Center-Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{9522C816-76C0-4C18-AAAD-0D4D9CF50C8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF5CCCB8-3EAD-4674-939A-6529E2509BBA}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="14_{56C020B2-A154-48CA-B7AA-0A5181D51BCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CFFB7C59-8163-42F8-A3E3-CDB3C963C3C4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{9D018150-ACE6-45E9-BEB1-34311369391D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{9D018150-ACE6-45E9-BEB1-34311369391D}"/>
   </bookViews>
   <sheets>
     <sheet name="customers" sheetId="3" r:id="rId1"/>
@@ -20,8 +20,8 @@
     <sheet name="pivots" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlcn.WorksheetConnection_Callcenteranalysis.xlsxcalls" hidden="1">calls[]</definedName>
-    <definedName name="_xlcn.WorksheetConnection_Callcenteranalysis.xlsxcustomers" hidden="1">customers[]</definedName>
+    <definedName name="_xlcn.WorksheetConnection_Callcenteranalysis.xlsxcalls1" hidden="1">calls[]</definedName>
+    <definedName name="_xlcn.WorksheetConnection_Callcenteranalysis.xlsxcustomers1" hidden="1">customers[]</definedName>
     <definedName name="ExternalData_1" localSheetId="2" hidden="1">'calls'!$A$1:$K$1001</definedName>
     <definedName name="ExternalData_2" localSheetId="2" hidden="1">'calls'!$M$1:$P$16</definedName>
     <definedName name="ExternalData_2" localSheetId="0" hidden="1">'customers'!$A$1:$D$16</definedName>
@@ -34,11 +34,11 @@
     <pivotCache cacheId="1" r:id="rId7"/>
     <pivotCache cacheId="2" r:id="rId8"/>
     <pivotCache cacheId="3" r:id="rId9"/>
-    <pivotCache cacheId="4" r:id="rId10"/>
-    <pivotCache cacheId="5" r:id="rId11"/>
-    <pivotCache cacheId="6" r:id="rId12"/>
-    <pivotCache cacheId="7" r:id="rId13"/>
-    <pivotCache cacheId="8" r:id="rId14"/>
+    <pivotCache cacheId="12" r:id="rId10"/>
+    <pivotCache cacheId="15" r:id="rId11"/>
+    <pivotCache cacheId="18" r:id="rId12"/>
+    <pivotCache cacheId="21" r:id="rId13"/>
+    <pivotCache cacheId="24" r:id="rId14"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{876F7934-8845-4945-9796-88D515C7AA90}">
@@ -60,8 +60,8 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{FCE2AD5D-F65C-4FA6-A056-5C36A1767C68}">
       <x15:dataModel>
         <x15:modelTables>
+          <x15:modelTable id="customers" name="customers" connection="WorksheetConnection_Call center analysis.xlsx!customers"/>
           <x15:modelTable id="calls" name="calls" connection="WorksheetConnection_Call center analysis.xlsx!calls"/>
-          <x15:modelTable id="customers" name="customers" connection="WorksheetConnection_Call center analysis.xlsx!customers"/>
         </x15:modelTables>
         <x15:modelRelationships>
           <x15:modelRelationship fromTable="calls" fromColumn="Customer ID" toTable="customers" toColumn="Customer ID"/>
@@ -121,7 +121,7 @@
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="calls" autoDelete="1">
-          <x15:rangePr sourceName="_xlcn.WorksheetConnection_Callcenteranalysis.xlsxcalls"/>
+          <x15:rangePr sourceName="_xlcn.WorksheetConnection_Callcenteranalysis.xlsxcalls1"/>
         </x15:connection>
       </ext>
     </extLst>
@@ -130,7 +130,7 @@
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="customers">
-          <x15:rangePr sourceName="_xlcn.WorksheetConnection_Callcenteranalysis.xlsxcustomers"/>
+          <x15:rangePr sourceName="_xlcn.WorksheetConnection_Callcenteranalysis.xlsxcustomers1"/>
         </x15:connection>
       </ext>
     </extLst>
@@ -3554,7 +3554,26 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="20">
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF8463"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -3675,7 +3694,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Call_Center_Performance_Dashboard.xlsx.xlsx]pivots!Monthly Trend</c:name>
+    <c:name>[Call_Center_Performance_Dashboard.xlsx]pivots!Monthly Trend</c:name>
     <c:fmtId val="2"/>
   </c:pivotSource>
   <c:chart>
@@ -4299,40 +4318,40 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>21</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>18</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>31</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20</c:v>
+                  <c:v>29</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8</c:v>
+                  <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>12</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>12</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>20</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>12</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>15</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4454,40 +4473,40 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>21</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>18</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>31</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20</c:v>
+                  <c:v>29</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8</c:v>
+                  <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>12</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>12</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>20</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>12</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>15</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4699,7 +4718,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Call_Center_Performance_Dashboard.xlsx.xlsx]pivots!Weekday trend</c:name>
+    <c:name>[Call_Center_Performance_Dashboard.xlsx]pivots!Weekday trend</c:name>
     <c:fmtId val="2"/>
   </c:pivotSource>
   <c:chart>
@@ -5001,25 +5020,25 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>27</c:v>
+                  <c:v>36</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>22</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>27</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>27</c:v>
+                  <c:v>23</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>27</c:v>
+                  <c:v>23</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>32</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>38</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5216,7 +5235,7 @@
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
-              <a:t>Calls</a:t>
+              <a:t>Amount</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -5450,7 +5469,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>18415</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>#N/A</c:v>
@@ -5462,7 +5481,7 @@
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>20104</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5631,7 +5650,7 @@
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
-              <a:t>Amount</a:t>
+              <a:t>Calls</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -5844,7 +5863,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>189</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>#N/A</c:v>
@@ -5856,7 +5875,7 @@
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>200</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6001,7 +6020,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Call_Center_Performance_Dashboard.xlsx.xlsx]pivots!Male female call</c:name>
+    <c:name>[Call_Center_Performance_Dashboard.xlsx]pivots!Male female call</c:name>
     <c:fmtId val="9"/>
   </c:pivotSource>
   <c:chart>
@@ -6914,7 +6933,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Call_Center_Performance_Dashboard.xlsx.xlsx]pivots!Rep satisfaction</c:name>
+    <c:name>[Call_Center_Performance_Dashboard.xlsx]pivots!Rep satisfaction</c:name>
     <c:fmtId val="13"/>
   </c:pivotSource>
   <c:chart>
@@ -7151,19 +7170,22 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>pivots!$A$53:$A$57</c:f>
+              <c:f>pivots!$A$53:$A$58</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>3</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>4</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>5</c:v>
                 </c:pt>
               </c:strCache>
@@ -7171,21 +7193,24 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>pivots!$B$53:$B$57</c:f>
+              <c:f>pivots!$B$53:$B$58</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>10</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>44</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>95</c:v>
+                  <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>51</c:v>
+                  <c:v>88</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>60</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11419,7 +11444,7 @@
               <a:latin typeface="Bahnschrift SemiLight SemiConde"/>
             </a:rPr>
             <a:pPr algn="ctr"/>
-            <a:t>200</a:t>
+            <a:t>189</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="1100">
             <a:solidFill>
@@ -11685,7 +11710,7 @@
               <a:latin typeface="Bahnschrift SemiLight SemiConde"/>
             </a:rPr>
             <a:pPr algn="ctr"/>
-            <a:t>$20,104</a:t>
+            <a:t>$18,415</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="1100">
             <a:solidFill>
@@ -12217,7 +12242,7 @@
               <a:latin typeface="Bahnschrift SemiLight SemiConde"/>
             </a:rPr>
             <a:pPr algn="ctr"/>
-            <a:t>18209</a:t>
+            <a:t>16834</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="1100">
             <a:solidFill>
@@ -12497,7 +12522,7 @@
               <a:latin typeface="Bahnschrift SemiLight SemiConde"/>
             </a:rPr>
             <a:pPr algn="ctr"/>
-            <a:t>51</a:t>
+            <a:t>60</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="1100">
             <a:solidFill>
@@ -13504,7 +13529,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="arnob" refreshedDate="46251.196906365738" backgroundQuery="1" createdVersion="7" refreshedVersion="7" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{CB87C1E4-0605-4DCA-9E03-1FBA280B49DB}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="arnob" refreshedDate="46253.142070138892" backgroundQuery="1" createdVersion="7" refreshedVersion="7" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{CB87C1E4-0605-4DCA-9E03-1FBA280B49DB}">
   <cacheSource type="external" connectionId="5"/>
   <cacheFields count="6">
     <cacheField name="[Measures].[Call Count]" caption="Call Count" numFmtId="0" hierarchy="17" level="32767"/>
@@ -13592,7 +13617,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="arnob" refreshedDate="46251.196906944446" backgroundQuery="1" createdVersion="7" refreshedVersion="7" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{8693693C-5F04-4D72-B469-FEDAAA202705}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="arnob" refreshedDate="46253.142074768519" backgroundQuery="1" createdVersion="7" refreshedVersion="7" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{8693693C-5F04-4D72-B469-FEDAAA202705}">
   <cacheSource type="external" connectionId="5"/>
   <cacheFields count="5">
     <cacheField name="[calls].[Representative].[Representative]" caption="Representative" numFmtId="0" hierarchy="3" level="1">
@@ -13713,7 +13738,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="arnob" refreshedDate="46251.196907407408" backgroundQuery="1" createdVersion="7" refreshedVersion="7" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{759D9313-94DA-44F7-A97E-34D8D8FE40CC}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="arnob" refreshedDate="46253.142079050929" backgroundQuery="1" createdVersion="7" refreshedVersion="7" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{759D9313-94DA-44F7-A97E-34D8D8FE40CC}">
   <cacheSource type="external" connectionId="5"/>
   <cacheFields count="3">
     <cacheField name="[calls].[Day of week].[Day of week]" caption="Day of week" numFmtId="0" hierarchy="8" level="1">
@@ -13797,12 +13822,12 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="arnob" refreshedDate="46251.196907754631" backgroundQuery="1" createdVersion="7" refreshedVersion="7" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{33C04E66-2D7C-4942-AE00-95174C3F3283}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="arnob" refreshedDate="46253.142083680556" backgroundQuery="1" createdVersion="7" refreshedVersion="7" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{33C04E66-2D7C-4942-AE00-95174C3F3283}">
   <cacheSource type="external" connectionId="5"/>
   <cacheFields count="1">
     <cacheField name="[calls].[Representative].[Representative]" caption="Representative" numFmtId="0" hierarchy="3" level="1">
       <sharedItems count="1">
-        <s v="R05"/>
+        <s v="R01"/>
       </sharedItems>
     </cacheField>
   </cacheFields>
@@ -13862,7 +13887,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition9.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="arnob" refreshedDate="46251.196908101854" backgroundQuery="1" createdVersion="7" refreshedVersion="7" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{24E00D43-5924-4397-B040-99B859E764D5}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="arnob" refreshedDate="46253.142088310182" backgroundQuery="1" createdVersion="7" refreshedVersion="7" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{24E00D43-5924-4397-B040-99B859E764D5}">
   <cacheSource type="external" connectionId="5"/>
   <cacheFields count="3">
     <cacheField name="[Measures].[Call Count]" caption="Call Count" numFmtId="0" hierarchy="17" level="32767"/>
@@ -13870,7 +13895,8 @@
       <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsString="0"/>
     </cacheField>
     <cacheField name="[calls].[Rating rounded].[Rating rounded]" caption="Rating rounded" numFmtId="0" hierarchy="10" level="1">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="2" maxValue="5" count="4">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="5" count="5">
+        <n v="1"/>
         <n v="2"/>
         <n v="3"/>
         <n v="4"/>
@@ -13879,10 +13905,11 @@
       <extLst>
         <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{4F2E5C28-24EA-4eb8-9CBF-B6C8F9C3D259}">
           <x15:cachedUniqueNames>
-            <x15:cachedUniqueName index="0" name="[calls].[Rating rounded].&amp;[2]"/>
-            <x15:cachedUniqueName index="1" name="[calls].[Rating rounded].&amp;[3]"/>
-            <x15:cachedUniqueName index="2" name="[calls].[Rating rounded].&amp;[4]"/>
-            <x15:cachedUniqueName index="3" name="[calls].[Rating rounded].&amp;[5]"/>
+            <x15:cachedUniqueName index="0" name="[calls].[Rating rounded].&amp;[1]"/>
+            <x15:cachedUniqueName index="1" name="[calls].[Rating rounded].&amp;[2]"/>
+            <x15:cachedUniqueName index="2" name="[calls].[Rating rounded].&amp;[3]"/>
+            <x15:cachedUniqueName index="3" name="[calls].[Rating rounded].&amp;[4]"/>
+            <x15:cachedUniqueName index="4" name="[calls].[Rating rounded].&amp;[5]"/>
           </x15:cachedUniqueNames>
         </ext>
       </extLst>
@@ -13953,400 +13980,6 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8A5B4F06-F1FD-4CDE-BD5C-DCEC3E33CA2E}" name="Summary pivot" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:E4" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="5">
-    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
-    <i i="3">
-      <x v="3"/>
-    </i>
-    <i i="4">
-      <x v="4"/>
-    </i>
-  </colItems>
-  <dataFields count="5">
-    <dataField fld="0" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField fld="2" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField fld="3" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField fld="4" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotHierarchies count="25">
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-  </pivotHierarchies>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <colHierarchiesUsage count="1">
-    <colHierarchyUsage hierarchyUsage="-2"/>
-  </colHierarchiesUsage>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
-      <x15:pivotTableUISettings sourceDataName="WorksheetConnection_Call center analysis.xlsx!calls">
-        <x15:activeTabTopLevelEntity name="[calls]"/>
-      </x15:pivotTableUISettings>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DDC153A1-84AB-4B96-8232-CFEC004A503D}" name="Selected Rep" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="B38:B39" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="1">
-    <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
-      <items count="1">
-        <item s="1" x="0"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="1">
-    <i>
-      <x/>
-    </i>
-  </rowItems>
-  <formats count="3">
-    <format dxfId="2">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="1">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="0">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
-  <pivotHierarchies count="25">
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-  </pivotHierarchies>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <rowHierarchiesUsage count="1">
-    <rowHierarchyUsage hierarchyUsage="3"/>
-  </rowHierarchiesUsage>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
-      <x15:pivotTableUISettings>
-        <x15:activeTabTopLevelEntity name="[calls]"/>
-      </x15:pivotTableUISettings>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{90226BDC-A20D-4FF5-BD2B-8EB3D6F63D7C}" name="PivotTable5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A29:C35" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="3">
-    <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="2">
-    <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField fld="2" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotHierarchies count="25">
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-  </pivotHierarchies>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <rowHierarchiesUsage count="1">
-    <rowHierarchyUsage hierarchyUsage="3"/>
-  </rowHierarchiesUsage>
-  <colHierarchiesUsage count="1">
-    <colHierarchyUsage hierarchyUsage="-2"/>
-  </colHierarchiesUsage>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
-      <x15:pivotTableUISettings sourceDataName="WorksheetConnection_Call center analysis.xlsx!calls">
-        <x15:activeTabTopLevelEntity name="[calls]"/>
-      </x15:pivotTableUISettings>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{94E8D690-8B5B-43D4-9F12-BD2AE2B2040F}" name="Weekday trend" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
-  <location ref="K4:L12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="3">
-    <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" sortType="ascending" defaultSubtotal="0" defaultAttributeDrillState="1">
-      <items count="7">
-        <item x="3"/>
-        <item x="1"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="2"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="8">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotHierarchies count="25">
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1">
-      <members count="1" level="1">
-        <member name="[calls].[Representative].&amp;[R05]"/>
-      </members>
-    </pivotHierarchy>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-  </pivotHierarchies>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <rowHierarchiesUsage count="1">
-    <rowHierarchyUsage hierarchyUsage="8"/>
-  </rowHierarchiesUsage>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
-      <x15:pivotTableUISettings sourceDataName="WorksheetConnection_Call center analysis.xlsx!calls">
-        <x15:activeTabTopLevelEntity name="[calls]"/>
-      </x15:pivotTableUISettings>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{84759B0E-7295-4341-A903-9D48985D3296}" name="PivotTable12" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" rowGrandTotals="0" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14">
   <location ref="A60:G79" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="4">
@@ -14525,25 +14158,28 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E1FCCD2F-746F-4F02-BE8B-CC8F2CDB063E}" name="Rep satisfaction" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14">
-  <location ref="A52:B57" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{94E8D690-8B5B-43D4-9F12-BD2AE2B2040F}" name="Weekday trend" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
+  <location ref="K4:L12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
+    <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" sortType="ascending" defaultSubtotal="0" defaultAttributeDrillState="1">
+      <items count="7">
+        <item x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="2"/>
+      </items>
+    </pivotField>
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
     <pivotField allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
-    <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-      </items>
-    </pivotField>
   </pivotFields>
   <rowFields count="1">
-    <field x="2"/>
+    <field x="0"/>
   </rowFields>
-  <rowItems count="5">
+  <rowItems count="8">
     <i>
       <x/>
     </i>
@@ -14555,6 +14191,252 @@
     </i>
     <i>
       <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotHierarchies count="25">
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1">
+      <members count="1" level="1">
+        <member name="[calls].[Representative].&amp;[R01]"/>
+      </members>
+    </pivotHierarchy>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+  </pivotHierarchies>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <rowHierarchiesUsage count="1">
+    <rowHierarchyUsage hierarchyUsage="8"/>
+  </rowHierarchiesUsage>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
+      <x15:pivotTableUISettings sourceDataName="WorksheetConnection_Call center analysis.xlsx!calls">
+        <x15:activeTabTopLevelEntity name="[calls]"/>
+      </x15:pivotTableUISettings>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{07E1EFDC-04BF-4BC8-82A5-B3FBEF219A25}" name="Male female call" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
+  <location ref="A43:D48" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="3">
+    <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField axis="axisCol" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
+      <items count="2">
+        <item x="0"/>
+        <item x="1"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="2"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="2">
+    <chartFormat chart="9" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotHierarchies count="25">
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+  </pivotHierarchies>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <rowHierarchiesUsage count="1">
+    <rowHierarchyUsage hierarchyUsage="15"/>
+  </rowHierarchiesUsage>
+  <colHierarchiesUsage count="1">
+    <colHierarchyUsage hierarchyUsage="13"/>
+  </colHierarchiesUsage>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
+      <x15:pivotTableUISettings>
+        <x15:activeTabTopLevelEntity name="[customers]"/>
+        <x15:activeTabTopLevelEntity name="[calls]"/>
+      </x15:pivotTableUISettings>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E1FCCD2F-746F-4F02-BE8B-CC8F2CDB063E}" name="Rep satisfaction" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14">
+  <location ref="A52:B58" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="3">
+    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
+    <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
     </i>
     <i t="grand">
       <x/>
@@ -14592,7 +14474,7 @@
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1">
       <members count="1" level="1">
-        <member name="[calls].[Representative].&amp;[R05]"/>
+        <member name="[calls].[Representative].&amp;[R01]"/>
       </members>
     </pivotHierarchy>
     <pivotHierarchy dragToData="1"/>
@@ -14638,8 +14520,200 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{90226BDC-A20D-4FF5-BD2B-8EB3D6F63D7C}" name="PivotTable5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A29:C35" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="3">
+    <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField fld="2" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotHierarchies count="25">
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+  </pivotHierarchies>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <rowHierarchiesUsage count="1">
+    <rowHierarchyUsage hierarchyUsage="3"/>
+  </rowHierarchiesUsage>
+  <colHierarchiesUsage count="1">
+    <colHierarchyUsage hierarchyUsage="-2"/>
+  </colHierarchiesUsage>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
+      <x15:pivotTableUISettings sourceDataName="WorksheetConnection_Call center analysis.xlsx!calls">
+        <x15:activeTabTopLevelEntity name="[calls]"/>
+      </x15:pivotTableUISettings>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DDC153A1-84AB-4B96-8232-CFEC004A503D}" name="Selected Rep" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="B38:B39" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="1">
+    <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
+      <items count="1">
+        <item s="1" x="0"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="1">
+    <i>
+      <x/>
+    </i>
+  </rowItems>
+  <formats count="3">
+    <format dxfId="5">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="4">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotHierarchies count="25">
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+  </pivotHierarchies>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <rowHierarchiesUsage count="1">
+    <rowHierarchyUsage hierarchyUsage="3"/>
+  </rowHierarchiesUsage>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
+      <x15:pivotTableUISettings>
+        <x15:activeTabTopLevelEntity name="[calls]"/>
+      </x15:pivotTableUISettings>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FCD6EAEE-2D8B-48C8-8FB8-90E20133CB52}" name="Monthly Trend" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FCD6EAEE-2D8B-48C8-8FB8-90E20133CB52}" name="Monthly Trend" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
   <location ref="A11:C24" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
@@ -14785,7 +14859,7 @@
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1">
       <members count="1" level="1">
-        <member name="[calls].[Representative].&amp;[R05]"/>
+        <member name="[calls].[Representative].&amp;[R01]"/>
       </members>
     </pivotHierarchy>
     <pivotHierarchy dragToData="1"/>
@@ -14842,137 +14916,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{07E1EFDC-04BF-4BC8-82A5-B3FBEF219A25}" name="Male female call" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
-  <location ref="A43:D48" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="3">
-    <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField axis="axisCol" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
-      <items count="2">
-        <item x="0"/>
-        <item x="1"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="2"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="2">
-    <chartFormat chart="9" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="2" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="9" format="5" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="2" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotHierarchies count="25">
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-  </pivotHierarchies>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <rowHierarchiesUsage count="1">
-    <rowHierarchyUsage hierarchyUsage="15"/>
-  </rowHierarchiesUsage>
-  <colHierarchiesUsage count="1">
-    <colHierarchyUsage hierarchyUsage="13"/>
-  </colHierarchiesUsage>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
-      <x15:pivotTableUISettings>
-        <x15:activeTabTopLevelEntity name="[customers]"/>
-        <x15:activeTabTopLevelEntity name="[calls]"/>
-      </x15:pivotTableUISettings>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7D00920D-317A-42D5-BC9C-71F0B3C5D41C}" name="Rep pivot" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7D00920D-317A-42D5-BC9C-71F0B3C5D41C}" name="Rep pivot" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A7:E8" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="6">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -15018,9 +14962,96 @@
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1">
       <members count="1" level="1">
-        <member name="[calls].[Representative].&amp;[R05]"/>
+        <member name="[calls].[Representative].&amp;[R01]"/>
       </members>
     </pivotHierarchy>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+  </pivotHierarchies>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <colHierarchiesUsage count="1">
+    <colHierarchyUsage hierarchyUsage="-2"/>
+  </colHierarchiesUsage>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
+      <x15:pivotTableUISettings sourceDataName="WorksheetConnection_Call center analysis.xlsx!calls">
+        <x15:activeTabTopLevelEntity name="[calls]"/>
+      </x15:pivotTableUISettings>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8A5B4F06-F1FD-4CDE-BD5C-DCEC3E33CA2E}" name="Summary pivot" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:E4" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="5">
+    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+    <i i="3">
+      <x v="3"/>
+    </i>
+    <i i="4">
+      <x v="4"/>
+    </i>
+  </colItems>
+  <dataFields count="5">
+    <dataField fld="0" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField fld="2" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField fld="3" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField fld="4" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotHierarchies count="25">
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
+    <pivotHierarchy dragToData="1"/>
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy dragToData="1"/>
@@ -15146,7 +15177,7 @@
         </level>
       </levels>
       <selections count="1">
-        <selection n="[calls].[Representative].&amp;[R05]"/>
+        <selection n="[calls].[Representative].&amp;[R01]"/>
       </selections>
     </olap>
   </data>
@@ -15169,10 +15200,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D5F76CE3-B50A-498A-8C20-803F7D268944}" name="customers" displayName="customers" ref="A1:D16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:D16" xr:uid="{D5F76CE3-B50A-498A-8C20-803F7D268944}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{DF3C8C46-B80C-4F62-B849-6E2C8E48618E}" uniqueName="1" name="Customer ID" queryTableFieldId="1" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{6F1AA242-07D5-4EAF-BF35-C599A4C7FC68}" uniqueName="2" name="Gedner" queryTableFieldId="2" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{DF3C8C46-B80C-4F62-B849-6E2C8E48618E}" uniqueName="1" name="Customer ID" queryTableFieldId="1" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{6F1AA242-07D5-4EAF-BF35-C599A4C7FC68}" uniqueName="2" name="Gedner" queryTableFieldId="2" dataDxfId="18"/>
     <tableColumn id="3" xr3:uid="{28E45CF5-95BC-4315-9048-716A3D74907D}" uniqueName="3" name="Age" queryTableFieldId="3"/>
-    <tableColumn id="4" xr3:uid="{2403355B-DE99-4B00-9CB3-12840C8DB946}" uniqueName="4" name="City" queryTableFieldId="4" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{2403355B-DE99-4B00-9CB3-12840C8DB946}" uniqueName="4" name="City" queryTableFieldId="4" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -15182,7 +15213,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6CF38917-483D-4CF0-910C-6B9C536C4BAA}" name="Assets" displayName="Assets" ref="A1:B6" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:B6" xr:uid="{6CF38917-483D-4CF0-910C-6B9C536C4BAA}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{74278F65-28BE-4E1B-8956-6D42DE9CB9C2}" uniqueName="1" name="Rep ID" queryTableFieldId="1" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{74278F65-28BE-4E1B-8956-6D42DE9CB9C2}" uniqueName="1" name="Rep ID" queryTableFieldId="1" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{5EE54E3C-F700-4BCD-BE0D-8D3CF15DA76C}" uniqueName="2" name="Rep Image" queryTableFieldId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -15193,16 +15224,16 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A4B3608E-B430-4E96-8C7D-9782FFD84484}" name="calls" displayName="calls" ref="A1:K1001" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:K1001" xr:uid="{A4B3608E-B430-4E96-8C7D-9782FFD84484}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{C96ED53A-C7AB-4DAA-8144-76D61643F4F3}" uniqueName="1" name="Call number" queryTableFieldId="1" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{8131FEE3-FA7B-437A-9DB2-F2FBF2CB2BB1}" uniqueName="2" name="Customer ID" queryTableFieldId="2" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{C96ED53A-C7AB-4DAA-8144-76D61643F4F3}" uniqueName="1" name="Call number" queryTableFieldId="1" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{8131FEE3-FA7B-437A-9DB2-F2FBF2CB2BB1}" uniqueName="2" name="Customer ID" queryTableFieldId="2" dataDxfId="14"/>
     <tableColumn id="3" xr3:uid="{491218FA-DA05-487A-8632-3DB9E58B1CDB}" uniqueName="3" name="Duration" queryTableFieldId="3"/>
-    <tableColumn id="4" xr3:uid="{9BEF716C-A937-4F5B-9851-BE108A8C6117}" uniqueName="4" name="Representative" queryTableFieldId="4" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{A2DC4A49-A101-4EBE-B7DE-9E5953259F5A}" uniqueName="5" name="Date of Call" queryTableFieldId="5" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{9BEF716C-A937-4F5B-9851-BE108A8C6117}" uniqueName="4" name="Representative" queryTableFieldId="4" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{A2DC4A49-A101-4EBE-B7DE-9E5953259F5A}" uniqueName="5" name="Date of Call" queryTableFieldId="5" dataDxfId="12"/>
     <tableColumn id="6" xr3:uid="{0ACA9E29-9B61-49FE-9AF0-9311729D19AB}" uniqueName="6" name="Purchase Amount" queryTableFieldId="6"/>
     <tableColumn id="7" xr3:uid="{5AF41280-BD17-4509-A697-A79F45C392D5}" uniqueName="7" name="Satisfaction Rating" queryTableFieldId="7"/>
     <tableColumn id="8" xr3:uid="{8CF5CF8B-4076-4427-A23D-C4485596DCB0}" uniqueName="8" name="FY" queryTableFieldId="8"/>
-    <tableColumn id="9" xr3:uid="{D0D63A6A-D6F1-4527-880E-9BAE8FF78BC7}" uniqueName="9" name="Day of week" queryTableFieldId="9" dataDxfId="8"/>
-    <tableColumn id="10" xr3:uid="{6EA70F58-1B02-40ED-B894-E175950FA48E}" uniqueName="10" name="Duration Bucket" queryTableFieldId="10" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{D0D63A6A-D6F1-4527-880E-9BAE8FF78BC7}" uniqueName="9" name="Day of week" queryTableFieldId="9" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{6EA70F58-1B02-40ED-B894-E175950FA48E}" uniqueName="10" name="Duration Bucket" queryTableFieldId="10" dataDxfId="10"/>
     <tableColumn id="11" xr3:uid="{B24CEF15-DFC9-4086-85C0-DFA91F02EA0E}" uniqueName="11" name="Rating rounded" queryTableFieldId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -15213,10 +15244,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BC704E26-0E79-4D55-8954-4B5F62E3477B}" name="customers4" displayName="customers4" ref="M1:P16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="M1:P16" xr:uid="{BC704E26-0E79-4D55-8954-4B5F62E3477B}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2A50C832-8FF1-4D93-B3D1-F687EBAA343F}" uniqueName="1" name="Customer ID" queryTableFieldId="1" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{02A5636B-7703-40B5-8640-1AF7FF18C818}" uniqueName="2" name="Gender" queryTableFieldId="2" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{2A50C832-8FF1-4D93-B3D1-F687EBAA343F}" uniqueName="1" name="Customer ID" queryTableFieldId="1" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{02A5636B-7703-40B5-8640-1AF7FF18C818}" uniqueName="2" name="Gender" queryTableFieldId="2" dataDxfId="8"/>
     <tableColumn id="3" xr3:uid="{C6F46C1E-C695-4462-AF6A-DE801CC30829}" uniqueName="3" name="Age" queryTableFieldId="3"/>
-    <tableColumn id="4" xr3:uid="{0E4221F3-8BF1-471F-9B1B-36FE597F4D16}" uniqueName="4" name="City" queryTableFieldId="4" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{0E4221F3-8BF1-471F-9B1B-36FE597F4D16}" uniqueName="4" name="City" queryTableFieldId="4" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -54500,7 +54531,8 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -54571,7 +54603,7 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
       <x14:slicerList>
-        <x14:slicer r:id="rId2"/>
+        <x14:slicer r:id="rId3"/>
       </x14:slicerList>
     </ext>
   </extLst>
@@ -54583,18 +54615,18 @@
   <dimension ref="A3:O79"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.75" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.875" bestFit="1" customWidth="1"/>
     <col min="13" max="14" width="9.375" customWidth="1"/>
     <col min="15" max="15" width="1.5" bestFit="1" customWidth="1"/>
     <col min="16" max="17" width="8.625" customWidth="1"/>
@@ -54715,7 +54747,7 @@
         <v>14</v>
       </c>
       <c r="L5" s="3">
-        <v>27</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -54723,7 +54755,7 @@
         <v>26</v>
       </c>
       <c r="L6" s="3">
-        <v>22</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -54746,30 +54778,30 @@
         <v>29</v>
       </c>
       <c r="L7" s="3">
-        <v>27</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="B8" s="4">
-        <v>20104</v>
+        <v>18415</v>
       </c>
       <c r="C8" s="5">
-        <v>18209</v>
+        <v>16834</v>
       </c>
       <c r="D8" s="6">
-        <v>3.8824999999999998</v>
+        <v>3.9227513227513247</v>
       </c>
       <c r="E8" s="5">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="K8" s="10" t="s">
         <v>44</v>
       </c>
       <c r="L8" s="3">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
@@ -54777,7 +54809,7 @@
         <v>48</v>
       </c>
       <c r="L9" s="3">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
@@ -54785,7 +54817,7 @@
         <v>56</v>
       </c>
       <c r="L10" s="3">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
@@ -54802,7 +54834,7 @@
         <v>59</v>
       </c>
       <c r="L11" s="3">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
@@ -54810,16 +54842,16 @@
         <v>1061</v>
       </c>
       <c r="B12" s="3">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C12" s="3">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="K12" s="10" t="s">
         <v>1060</v>
       </c>
       <c r="L12" s="3">
-        <v>200</v>
+        <v>189</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
@@ -54827,10 +54859,10 @@
         <v>1062</v>
       </c>
       <c r="B13" s="3">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C13" s="3">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
@@ -54838,10 +54870,10 @@
         <v>1063</v>
       </c>
       <c r="B14" s="3">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C14" s="3">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
@@ -54849,10 +54881,10 @@
         <v>1064</v>
       </c>
       <c r="B15" s="3">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C15" s="3">
-        <v>20</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
@@ -54860,10 +54892,10 @@
         <v>1065</v>
       </c>
       <c r="B16" s="3">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C16" s="3">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
@@ -54871,10 +54903,10 @@
         <v>1066</v>
       </c>
       <c r="B17" s="3">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C17" s="3">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
@@ -54882,10 +54914,10 @@
         <v>1067</v>
       </c>
       <c r="B18" s="3">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C18" s="3">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
@@ -54904,10 +54936,10 @@
         <v>1069</v>
       </c>
       <c r="B20" s="3">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="C20" s="3">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
@@ -54926,10 +54958,10 @@
         <v>1071</v>
       </c>
       <c r="B22" s="3">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C22" s="3">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
@@ -54937,10 +54969,10 @@
         <v>1072</v>
       </c>
       <c r="B23" s="3">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C23" s="3">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="O23" t="s">
         <v>1058</v>
@@ -54951,10 +54983,10 @@
         <v>1060</v>
       </c>
       <c r="B24" s="3">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="C24" s="3">
-        <v>200</v>
+        <v>189</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
@@ -54997,17 +55029,17 @@
       <c r="H29" s="11">
         <v>18415</v>
       </c>
-      <c r="I29" t="e">
+      <c r="I29">
         <f>IF(F29=$L$29,G29,NA())</f>
-        <v>#N/A</v>
-      </c>
-      <c r="J29" t="e">
+        <v>189</v>
+      </c>
+      <c r="J29">
         <f>IF((F29=$L$29),H29,NA())</f>
-        <v>#N/A</v>
+        <v>18415</v>
       </c>
       <c r="L29" t="str">
         <f>B39</f>
-        <v>R05</v>
+        <v>R01</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
@@ -55113,13 +55145,13 @@
       <c r="H33" s="11">
         <v>20104</v>
       </c>
-      <c r="I33">
+      <c r="I33" t="e">
         <f t="shared" si="0"/>
-        <v>200</v>
-      </c>
-      <c r="J33">
+        <v>#N/A</v>
+      </c>
+      <c r="J33" t="e">
         <f t="shared" si="1"/>
-        <v>20104</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
@@ -55151,7 +55183,7 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B39" s="12" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
@@ -55242,42 +55274,50 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B53" s="3">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B54" s="3">
-        <v>44</v>
+        <v>9</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B55" s="3">
-        <v>95</v>
+        <v>31</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="10">
+        <v>4</v>
+      </c>
+      <c r="B56" s="3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" s="10">
         <v>5</v>
       </c>
-      <c r="B56" s="3">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A57" s="10" t="s">
+      <c r="B57" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" s="10" t="s">
         <v>1060</v>
       </c>
-      <c r="B57" s="3">
-        <v>200</v>
+      <c r="B58" s="3">
+        <v>189</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>